<commit_message>
Checked and updated the skill extractor
</commit_message>
<xml_diff>
--- a/compare_skill.xlsx
+++ b/compare_skill.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/h3ng/Documents/Projects/Job Matcher/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A154A15-FB99-D941-8FE9-FED42176F705}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7905C89-0C86-B24A-8CB9-9DD1E8FAD4B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38400" yWindow="1300" windowWidth="38400" windowHeight="21600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4300" yWindow="680" windowWidth="29900" windowHeight="19660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1095,6 +1095,7 @@
   <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
+    <col min="1" max="1" width="23" customWidth="1"/>
     <col min="2" max="2" width="65.1640625" style="1" customWidth="1"/>
     <col min="3" max="3" width="88" customWidth="1"/>
   </cols>

</xml_diff>